<commit_message>
Split property JV into JV-001 Cairnsford purchase and JV-002 Strensall remortgage
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UszXj8jDKmjemVNstTQPa2
</commit_message>
<xml_diff>
--- a/data/Completion_Statements.xlsx
+++ b/data/Completion_Statements.xlsx
@@ -8,9 +8,10 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="JV-001 Property Purchase" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Strensall Remortgage" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Cairnsford Purchase" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="JV-001 Cairnsford Purchase" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="JV-002 Strensall Remortgage" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Strensall Remortgage" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Cairnsford Purchase" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="124">
   <si>
     <t xml:space="preserve">Alino Property Ltd</t>
   </si>
@@ -45,7 +46,7 @@
     <t xml:space="preserve">Narration</t>
   </si>
   <si>
-    <t xml:space="preserve">Purchase of 36 Cairnsford Road, Leicester LE2 6GF, funded by a Together Commercial mortgage, the remortgage of 30 Strensall Road, and funds from Alvine Tchega and Kakmeni (per both completion statements).</t>
+    <t xml:space="preserve">Purchase of 36 Cairnsford Road, Leicester LE2 6GF (DWS Legal completion statement). Funded by a Together Commercial mortgage, the 30 Strensall remortgage proceeds (via solicitor clearing, see JV-002), Alvine Tchega and Kakmeni.</t>
   </si>
   <si>
     <t xml:space="preserve">Line</t>
@@ -96,12 +97,6 @@
     <t xml:space="preserve">Cairnsford: mortgage admin, lender sols, policy, MR01, insolvency indemnity</t>
   </si>
   <si>
-    <t xml:space="preserve">Remortgage costs – 30 Strensall Rd, incl. VAT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strensall: all 13 fee lines</t>
-  </si>
-  <si>
     <t xml:space="preserve">Mortgage – Together Commercial (Cairnsford)</t>
   </si>
   <si>
@@ -111,6 +106,90 @@
     <t xml:space="preserve">Cairnsford: Mortgage advance</t>
   </si>
   <si>
+    <t xml:space="preserve">Solicitor clearing – DWS Legal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 Strensall remortgage proceeds applied to purchase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cairnsford: Proceeds from 30 Strensall (clears JV-002 line 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Director's loan – Alvine Tchega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funds introduced 14/07/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cairnsford: Money from client – Alvine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Money on account paid to solicitors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cairnsford: Money on Account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan – Kakmeni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cairnsford: Money from client – Kakmeni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Totals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difference (must be 0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Green figures are formulas linked to the line items on the 'Cairnsford Purchase' sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Total cost of 36 Cairnsford Rd = lines 1–3 (£499,943.94). VAT on fees is included because the company is assumed not to be VAT-registered.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Line 5: Together's solicitors paid the loan direct to DWS, so it never went through the bank. This line records the loan the company owes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Line 6 credits solicitor clearing with the Strensall proceeds. JV-002 line 1 debits the same amount, so clearing nets to nil.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Lender fees (line 4) are posted to the P&amp;L as a finance cost. Under FRS 102 they can instead be netted against the loan and spread over its term.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Alvine's funds are treated as the director's loan account and Kakmeni's £38,000 as a loan. Change these if they were share capital or another arrangement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prepared by:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewed by:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Posted (date):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JV-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remortgage of 30 Strensall Road, Leicester LE2 9FT (completion statement ref 1093081). Together Commercial advance less costs; the net £131,958.00 was paid to DWS Legal for the 36 Cairnsford purchase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remortgage proceeds held by solicitor for Cairnsford purchase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strensall: Balance due on completion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remortgage costs – 30 Strensall Rd, incl. VAT (13 items)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strensall: all fee lines</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mortgage – Together Commercial (Strensall)</t>
   </si>
   <si>
@@ -120,61 +199,28 @@
     <t xml:space="preserve">Strensall: Mortgage advance</t>
   </si>
   <si>
-    <t xml:space="preserve">Director's loan – Alvine Tchega</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Funds introduced 14/07/2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cairnsford: Money from client – Alvine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Money on account paid to solicitors (£400 + £100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Both: Money on account</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loan – Kakmeni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cairnsford: Money from client – Kakmeni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Totals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Difference (must be 0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Green figures are formulas linked to the line items on the two statement sheets in this workbook.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. The 30 Strensall balance of £131,958.00 was paid out on the Strensall statement and received on the Cairnsford statement. It nets to nil, so it is not posted.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Total cost of 36 Cairnsford Rd = lines 1–3. VAT on fees is included because the company is assumed not to be VAT-registered.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Lender and remortgage fees (lines 4–5) are posted to Loan arrangement fees (P&amp;L finance cost). Under FRS 102 they can instead be netted against the loans and spread over the loan term.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Mortgages are recorded at the net advance shown on the statements. The gross loans per the Together Commercial offers may be higher by the lender's solicitor fees.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Alvine's funds are treated as the director's loan account and Kakmeni's £38,000 as a loan. Change these if they were share capital or another arrangement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepared by:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reviewed by:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Posted (date):</t>
+    <t xml:space="preserve">Money on account 08/04/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strensall: Money on account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Green figures are formulas linked to the line items on the 'Strensall Remortgage' sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Line 1: the £131,958.00 balance due was not paid to the company's bank. It went straight into the Cairnsford purchase, so it is debited to solicitor clearing and cleared by JV-001 line 6.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Line 3: Together's advance is recorded net of the lender's solicitor fees deducted before it reached the company's solicitor. The offer letter will show the gross loan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Remortgage costs (line 2) are posted to the P&amp;L as a finance cost. They can instead be netted against the loan and spread over its term.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. 30 Strensall Road itself is not in this JV because it was already owned. Its cost should already be in the books; it is not in the records provided.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Check: JV-001 line 6 credit = JV-002 line 1 debit, so solicitor clearing nets to £0.00.</t>
   </si>
   <si>
     <t xml:space="preserve">Completion Statement</t>
@@ -856,12 +902,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="58"/>
   </cols>
@@ -1013,18 +1059,18 @@
         <v>5</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <f aca="false">'Strensall Remortgage'!E10+'Strensall Remortgage'!E11+'Strensall Remortgage'!E12+'Strensall Remortgage'!E13+'Strensall Remortgage'!E14+'Strensall Remortgage'!E15+'Strensall Remortgage'!E16+'Strensall Remortgage'!E17+'Strensall Remortgage'!E18+'Strensall Remortgage'!E19+'Strensall Remortgage'!E20+'Strensall Remortgage'!E21+'Strensall Remortgage'!E22</f>
-        <v>1670</v>
-      </c>
-      <c r="E13" s="8"/>
+        <v>25</v>
+      </c>
+      <c r="D13" s="8"/>
+      <c r="E13" s="7" t="n">
+        <f aca="false">'Cairnsford Purchase'!B10</f>
+        <v>311938.6</v>
+      </c>
       <c r="F13" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1032,18 +1078,18 @@
         <v>6</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="7" t="n">
-        <f aca="false">'Cairnsford Purchase'!B10</f>
-        <v>311938.6</v>
+        <f aca="false">'Cairnsford Purchase'!B11</f>
+        <v>131958</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1051,18 +1097,18 @@
         <v>7</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="7" t="n">
-        <f aca="false">'Strensall Remortgage'!B8</f>
-        <v>133528</v>
+        <f aca="false">'Cairnsford Purchase'!B12</f>
+        <v>18362.34</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1070,15 +1116,15 @@
         <v>8</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>33</v>
       </c>
       <c r="D16" s="8"/>
       <c r="E16" s="7" t="n">
-        <f aca="false">'Cairnsford Purchase'!B12</f>
-        <v>18362.34</v>
+        <f aca="false">'Cairnsford Purchase'!B9</f>
+        <v>400</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>34</v>
@@ -1089,73 +1135,64 @@
         <v>9</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D17" s="8"/>
       <c r="E17" s="7" t="n">
-        <f aca="false">'Cairnsford Purchase'!B9+'Strensall Remortgage'!B9</f>
-        <v>500</v>
+        <f aca="false">'Cairnsford Purchase'!B13</f>
+        <v>38000</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="7" t="n">
-        <f aca="false">'Cairnsford Purchase'!B13</f>
-        <v>38000</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>38</v>
+      <c r="D18" s="9" t="n">
+        <f aca="false">SUM(D9:D17)</f>
+        <v>500658.94</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <f aca="false">SUM(E9:E17)</f>
+        <v>500658.94</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C19" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <f aca="false">ROUND(D18-E18,2)</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="3" t="str">
+        <f aca="false">IF(D19=0,"Balanced","NOT BALANCED")</f>
+        <v>Balanced</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D19" s="9" t="n">
-        <f aca="false">SUM(D9:D18)</f>
-        <v>502328.94</v>
-      </c>
-      <c r="E19" s="9" t="n">
-        <f aca="false">SUM(E9:E18)</f>
-        <v>502328.94</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C20" s="3" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D20" s="10" t="n">
-        <f aca="false">ROUND(D19-E19,2)</f>
-        <v>0</v>
-      </c>
-      <c r="E20" s="3" t="str">
-        <f aca="false">IF(D20=0,"Balanced","NOT BALANCED")</f>
-        <v>Balanced</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
@@ -1165,7 +1202,7 @@
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
@@ -1175,7 +1212,7 @@
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
@@ -1185,7 +1222,7 @@
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
@@ -1195,7 +1232,7 @@
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
@@ -1203,45 +1240,35 @@
       <c r="E27" s="11"/>
       <c r="F27" s="11"/>
     </row>
-    <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B31" s="12"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B6:F6"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A25:F25"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A28:F28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1258,349 +1285,279 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="D9" s="7" t="n">
+        <f aca="false">'Strensall Remortgage'!E25</f>
+        <v>131958</v>
+      </c>
+      <c r="E9" s="8"/>
+      <c r="F9" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="D10" s="7" t="n">
+        <f aca="false">'Strensall Remortgage'!E10+'Strensall Remortgage'!E11+'Strensall Remortgage'!E12+'Strensall Remortgage'!E13+'Strensall Remortgage'!E14+'Strensall Remortgage'!E15+'Strensall Remortgage'!E16+'Strensall Remortgage'!E17+'Strensall Remortgage'!E18+'Strensall Remortgage'!E19+'Strensall Remortgage'!E20+'Strensall Remortgage'!E21+'Strensall Remortgage'!E22</f>
+        <v>1670</v>
+      </c>
+      <c r="E10" s="8"/>
+      <c r="F10" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-    </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="C11" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="D11" s="8"/>
+      <c r="E11" s="7" t="n">
+        <f aca="false">'Strensall Remortgage'!B8</f>
+        <v>133528</v>
+      </c>
+      <c r="F11" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="13" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="D12" s="8"/>
+      <c r="E12" s="7" t="n">
+        <f aca="false">'Strensall Remortgage'!B9</f>
+        <v>100</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <f aca="false">SUM(D9:D12)</f>
+        <v>133628</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <f aca="false">SUM(E9:E12)</f>
+        <v>133628</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <f aca="false">ROUND(D13-E13,2)</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="3" t="str">
+        <f aca="false">IF(D14=0,"Balanced","NOT BALANCED")</f>
+        <v>Balanced</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="14" t="n">
-        <v>133528</v>
-      </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="8"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+    </row>
+    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="8"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+    </row>
+    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14" t="n">
-        <v>650</v>
-      </c>
-      <c r="D10" s="14" t="n">
-        <v>130</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <f aca="false">C10+D10</f>
-        <v>780</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+    </row>
+    <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14" t="n">
-        <v>35</v>
-      </c>
-      <c r="D11" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="E11" s="8" t="n">
-        <f aca="false">C11+D11</f>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+    </row>
+    <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14" t="n">
-        <v>200</v>
-      </c>
-      <c r="D12" s="14" t="n">
-        <v>40</v>
-      </c>
-      <c r="E12" s="8" t="n">
-        <f aca="false">C12+D12</f>
-        <v>240</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+    </row>
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14" t="n">
-        <v>300</v>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>60</v>
-      </c>
-      <c r="E13" s="8" t="n">
-        <f aca="false">C13+D13</f>
-        <v>360</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14" t="n">
-        <v>29</v>
-      </c>
-      <c r="D14" s="14"/>
-      <c r="E14" s="8" t="n">
-        <f aca="false">C14+D14</f>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14" t="n">
-        <v>18</v>
-      </c>
-      <c r="D15" s="14"/>
-      <c r="E15" s="8" t="n">
-        <f aca="false">C15+D15</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14" t="n">
-        <v>45</v>
-      </c>
-      <c r="D16" s="14"/>
-      <c r="E16" s="8" t="n">
-        <f aca="false">C16+D16</f>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14" t="n">
-        <v>14</v>
-      </c>
-      <c r="D17" s="14"/>
-      <c r="E17" s="8" t="n">
-        <f aca="false">C17+D17</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="D18" s="14"/>
-      <c r="E18" s="8" t="n">
-        <f aca="false">C18+D18</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14" t="n">
-        <v>45</v>
-      </c>
-      <c r="D19" s="14"/>
-      <c r="E19" s="8" t="n">
-        <f aca="false">C19+D19</f>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14" t="n">
-        <v>15</v>
-      </c>
-      <c r="D20" s="14"/>
-      <c r="E20" s="8" t="n">
-        <f aca="false">C20+D20</f>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14" t="n">
-        <v>15</v>
-      </c>
-      <c r="D21" s="14"/>
-      <c r="E21" s="8" t="n">
-        <f aca="false">C21+D21</f>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14" t="n">
-        <v>60</v>
-      </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="8" t="n">
-        <f aca="false">C22+D22</f>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="B23" s="15" t="n">
-        <f aca="false">SUM(B8:B22)</f>
-        <v>133628</v>
-      </c>
-      <c r="C23" s="15" t="n">
-        <f aca="false">SUM(C8:C22)</f>
-        <v>1433</v>
-      </c>
-      <c r="D23" s="15" t="n">
-        <f aca="false">SUM(D8:D22)</f>
-        <v>237</v>
-      </c>
-      <c r="E23" s="15" t="n">
-        <f aca="false">SUM(E8:E22)</f>
-        <v>1670</v>
-      </c>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="E25" s="16" t="n">
-        <f aca="false">B23-E23</f>
-        <v>131958</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="B28" s="18" t="n">
-        <v>133628</v>
-      </c>
-      <c r="C28" s="3" t="str">
-        <f aca="false">IF(ROUND(B23-B28,2)=0,"Agrees","DIFFERENCE "&amp;TEXT(B23-B28,"#,##0.00"))</f>
-        <v>Agrees</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="B29" s="18" t="n">
-        <v>1670</v>
-      </c>
-      <c r="C29" s="3" t="str">
-        <f aca="false">IF(ROUND(E23-B29,2)=0,"Agrees","DIFFERENCE "&amp;TEXT(E23-B29,"#,##0.00"))</f>
-        <v>Agrees</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="B30" s="18" t="n">
-        <v>131958</v>
-      </c>
-      <c r="C30" s="3" t="str">
-        <f aca="false">IF(ROUND(E25-B30,2)=0,"Agrees","DIFFERENCE "&amp;TEXT(E25-B30,"#,##0.00"))</f>
-        <v>Agrees</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="19" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="19" t="s">
-        <v>82</v>
-      </c>
+      <c r="A25" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="12"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" s="12"/>
     </row>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A22:F22"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1616,6 +1573,364 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>133528</v>
+      </c>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="8"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14" t="n">
+        <v>650</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>130</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <f aca="false">C10+D10</f>
+        <v>780</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14" t="n">
+        <v>35</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <f aca="false">C11+D11</f>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <f aca="false">C12+D12</f>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <f aca="false">C13+D13</f>
+        <v>360</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14" t="n">
+        <v>29</v>
+      </c>
+      <c r="D14" s="14"/>
+      <c r="E14" s="8" t="n">
+        <f aca="false">C14+D14</f>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="14"/>
+      <c r="C15" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="D15" s="14"/>
+      <c r="E15" s="8" t="n">
+        <f aca="false">C15+D15</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="D16" s="14"/>
+      <c r="E16" s="8" t="n">
+        <f aca="false">C16+D16</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="D17" s="14"/>
+      <c r="E17" s="8" t="n">
+        <f aca="false">C17+D17</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" s="14"/>
+      <c r="E18" s="8" t="n">
+        <f aca="false">C18+D18</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14" t="n">
+        <v>45</v>
+      </c>
+      <c r="D19" s="14"/>
+      <c r="E19" s="8" t="n">
+        <f aca="false">C19+D19</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D20" s="14"/>
+      <c r="E20" s="8" t="n">
+        <f aca="false">C20+D20</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D21" s="14"/>
+      <c r="E21" s="8" t="n">
+        <f aca="false">C21+D21</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D22" s="14"/>
+      <c r="E22" s="8" t="n">
+        <f aca="false">C22+D22</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" s="15" t="n">
+        <f aca="false">SUM(B8:B22)</f>
+        <v>133628</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <f aca="false">SUM(C8:C22)</f>
+        <v>1433</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <f aca="false">SUM(D8:D22)</f>
+        <v>237</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <f aca="false">SUM(E8:E22)</f>
+        <v>1670</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E25" s="16" t="n">
+        <f aca="false">B23-E23</f>
+        <v>131958</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B28" s="18" t="n">
+        <v>133628</v>
+      </c>
+      <c r="C28" s="3" t="str">
+        <f aca="false">IF(ROUND(B23-B28,2)=0,"Agrees","DIFFERENCE "&amp;TEXT(B23-B28,"#,##0.00"))</f>
+        <v>Agrees</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="B29" s="18" t="n">
+        <v>1670</v>
+      </c>
+      <c r="C29" s="3" t="str">
+        <f aca="false">IF(ROUND(E23-B29,2)=0,"Agrees","DIFFERENCE "&amp;TEXT(E23-B29,"#,##0.00"))</f>
+        <v>Agrees</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B30" s="18" t="n">
+        <v>131958</v>
+      </c>
+      <c r="C30" s="3" t="str">
+        <f aca="false">IF(ROUND(E25-B30,2)=0,"Agrees","DIFFERENCE "&amp;TEXT(E25-B30,"#,##0.00"))</f>
+        <v>Agrees</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19" t="s">
+        <v>97</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1627,49 +1942,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B8" s="14"/>
       <c r="C8" s="14" t="n">
@@ -1683,7 +1998,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>400</v>
@@ -1694,7 +2009,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>311938.6</v>
@@ -1705,7 +2020,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="B11" s="14" t="n">
         <v>131958</v>
@@ -1716,7 +2031,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="B12" s="14" t="n">
         <v>18362.34</v>
@@ -1727,7 +2042,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="B13" s="14" t="n">
         <v>38000</v>
@@ -1738,7 +2053,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="14" t="n">
@@ -1754,7 +2069,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="B15" s="14"/>
       <c r="C15" s="14" t="n">
@@ -1770,7 +2085,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="14" t="n">
@@ -1786,7 +2101,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="14" t="n">
@@ -1802,7 +2117,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="B18" s="14"/>
       <c r="C18" s="14" t="n">
@@ -1818,7 +2133,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="B19" s="14"/>
       <c r="C19" s="14" t="n">
@@ -1834,7 +2149,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="B20" s="14"/>
       <c r="C20" s="14" t="n">
@@ -1850,7 +2165,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="B21" s="14"/>
       <c r="C21" s="14" t="n">
@@ -1864,7 +2179,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="B22" s="14"/>
       <c r="C22" s="14" t="n">
@@ -1878,7 +2193,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="B23" s="14"/>
       <c r="C23" s="14" t="n">
@@ -1892,7 +2207,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="14" t="n">
@@ -1906,7 +2221,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="14" t="n">
@@ -1920,7 +2235,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="B26" s="14"/>
       <c r="C26" s="14" t="n">
@@ -1934,7 +2249,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="B27" s="14"/>
       <c r="C27" s="14" t="n">
@@ -1948,7 +2263,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="14" t="n">
@@ -1962,7 +2277,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="14" t="n">
@@ -1976,7 +2291,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="14" t="n">
@@ -1990,7 +2305,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="B31" s="14"/>
       <c r="C31" s="14" t="n">
@@ -2004,7 +2319,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="B32" s="15" t="n">
         <f aca="false">SUM(B8:B31)</f>
@@ -2025,7 +2340,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="E34" s="16" t="n">
         <f aca="false">B32-E32</f>
@@ -2034,12 +2349,12 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="17" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="B37" s="18" t="n">
         <v>500658.94</v>
@@ -2051,7 +2366,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="17" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="B38" s="18" t="n">
         <v>500658.94</v>
@@ -2063,7 +2378,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="B39" s="18" t="n">
         <v>0</v>
@@ -2075,12 +2390,12 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="19" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="19" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>